<commit_message>
Actualización Ejercicio 3b: Inclusión de test de proactividad y métricas actualizadas
</commit_message>
<xml_diff>
--- a/resultados/Evaluación.xlsx
+++ b/resultados/Evaluación.xlsx
@@ -1549,7 +1549,7 @@
         <v>0.0</v>
       </c>
       <c r="H34" s="15">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="35">
@@ -1589,7 +1589,7 @@
         <v>0.0</v>
       </c>
       <c r="H36" s="15">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="37">
@@ -1671,7 +1671,7 @@
         <v>0.0</v>
       </c>
       <c r="H40" s="15">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="41">

</xml_diff>